<commit_message>
Objective 1 Succesfully completed
</commit_message>
<xml_diff>
--- a/Imp_sheet.xlsx
+++ b/Imp_sheet.xlsx
@@ -9,10 +9,11 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12210"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12210" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Modified_DL" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="157">
   <si>
     <t xml:space="preserve">         per-class IoU → cls0=0.468  cls1=0.010  cls2=0.555</t>
   </si>
@@ -282,6 +283,219 @@
   </si>
   <si>
     <t>Epoch 027 | train_loss=0.4282 | val_loss=0.7186 | val_mIoU=0.3443 | val_mF1=0.4571 | val_acc=0.6380</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  81,769 validation points loaded</t>
+  </si>
+  <si>
+    <t>Label values – train: [0, 1, 2]  |  val: [0, 1, 2]</t>
+  </si>
+  <si>
+    <t>Device: cpu</t>
+  </si>
+  <si>
+    <t>Using Combined Loss (Focal γ=2.0 + Dice w=0.3)</t>
+  </si>
+  <si>
+    <t>Epoch 001 | lr=2.08e-04 | train_loss=0.6305 | val_loss=1.0875 | val_mIoU=0.1384 | val_mF1=0.1959 | val_acc=0.4145</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.001  cls1=0.000  cls2=0.414</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         → New best mIoU: 0.1384  (best.pt saved)</t>
+  </si>
+  <si>
+    <t>Epoch 002 | lr=4.06e-04 | train_loss=0.5169 | val_loss=0.8752 | val_mIoU=0.1706 | val_mF1=0.2257 | val_acc=0.5117</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.512  cls1=0.000  cls2=0.000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         → New best mIoU: 0.1706  (best.pt saved)</t>
+  </si>
+  <si>
+    <t>Epoch 003 | lr=6.04e-04 | train_loss=0.4433 | val_loss=1.8911 | val_mIoU=0.1709 | val_mF1=0.2259 | val_acc=0.5126</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.513  cls1=0.000  cls2=0.000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         → New best mIoU: 0.1709  (best.pt saved)</t>
+  </si>
+  <si>
+    <t>Epoch 004 | lr=8.02e-04 | train_loss=0.4268 | val_loss=0.7401 | val_mIoU=0.1708 | val_mF1=0.2259 | val_acc=0.5124</t>
+  </si>
+  <si>
+    <t>Epoch 005 | lr=1.00e-03 | train_loss=0.4129 | val_loss=0.7007 | val_mIoU=0.1721 | val_mF1=0.2325 | val_acc=0.5046</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.501  cls1=0.000  cls2=0.015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         → New best mIoU: 0.1721  (best.pt saved)</t>
+  </si>
+  <si>
+    <t>Epoch 006 | lr=1.00e-03 | train_loss=0.4135 | val_loss=0.4696 | val_mIoU=0.2723 | val_mF1=0.3866 | val_acc=0.5601</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.420  cls1=0.000  cls2=0.397</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         → New best mIoU: 0.2723  (best.pt saved)</t>
+  </si>
+  <si>
+    <t>Epoch 007 | lr=9.99e-04 | train_loss=0.4141 | val_loss=0.4708 | val_mIoU=0.1445 | val_mF1=0.2077 | val_acc=0.4203</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.019  cls1=0.000  cls2=0.415</t>
+  </si>
+  <si>
+    <t>Epoch 008 | lr=9.98e-04 | train_loss=0.4101 | val_loss=0.4618 | val_mIoU=0.2419 | val_mF1=0.3509 | val_acc=0.5219</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.275  cls1=0.000  cls2=0.451</t>
+  </si>
+  <si>
+    <t>Epoch 009 | lr=9.96e-04 | train_loss=0.3964 | val_loss=0.4615 | val_mIoU=0.1385 | val_mF1=0.1957 | val_acc=0.4156</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.000  cls1=0.000  cls2=0.416</t>
+  </si>
+  <si>
+    <t>Epoch 010 | lr=9.93e-04 | train_loss=0.4058 | val_loss=0.4778 | val_mIoU=0.1708 | val_mF1=0.2259 | val_acc=0.5124</t>
+  </si>
+  <si>
+    <t>Epoch 011 | lr=9.90e-04 | train_loss=0.4000 | val_loss=0.4559 | val_mIoU=0.2984 | val_mF1=0.4115 | val_acc=0.5963</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.405  cls1=0.000  cls2=0.491</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         → New best mIoU: 0.2984  (best.pt saved)</t>
+  </si>
+  <si>
+    <t>Epoch 012 | lr=9.87e-04 | train_loss=0.3940 | val_loss=0.4652 | val_mIoU=0.1449 | val_mF1=0.2092 | val_acc=0.4190</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.022  cls1=0.000  cls2=0.412</t>
+  </si>
+  <si>
+    <t>Epoch 013 | lr=9.83e-04 | train_loss=0.3910 | val_loss=0.4609 | val_mIoU=0.1693 | val_mF1=0.2577 | val_acc=0.4292</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.120  cls1=0.000  cls2=0.388</t>
+  </si>
+  <si>
+    <t>Epoch 014 | lr=9.78e-04 | train_loss=0.3809 | val_loss=0.4547 | val_mIoU=0.1893 | val_mF1=0.2880 | val_acc=0.4512</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.180  cls1=0.000  cls2=0.387</t>
+  </si>
+  <si>
+    <t>Epoch 015 | lr=9.73e-04 | train_loss=0.3877 | val_loss=0.4906 | val_mIoU=0.2265 | val_mF1=0.3291 | val_acc=0.5187</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.466  cls1=0.000  cls2=0.213</t>
+  </si>
+  <si>
+    <t>Epoch 016 | lr=9.68e-04 | train_loss=0.3865 | val_loss=0.4625 | val_mIoU=0.2299 | val_mF1=0.3411 | val_acc=0.4993</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.306  cls1=0.000  cls2=0.384</t>
+  </si>
+  <si>
+    <t>Epoch 017 | lr=9.62e-04 | train_loss=0.3987 | val_loss=0.4795 | val_mIoU=0.2323 | val_mF1=0.3445 | val_acc=0.4980</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.347  cls1=0.000  cls2=0.350</t>
+  </si>
+  <si>
+    <t>Epoch 018 | lr=9.55e-04 | train_loss=0.3908 | val_loss=0.4580 | val_mIoU=0.2068 | val_mF1=0.3121 | val_acc=0.4718</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.232  cls1=0.000  cls2=0.388</t>
+  </si>
+  <si>
+    <t>Epoch 019 | lr=9.48e-04 | train_loss=0.3805 | val_loss=0.4832 | val_mIoU=0.2216 | val_mF1=0.3314 | val_acc=0.4879</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.285  cls1=0.000  cls2=0.380</t>
+  </si>
+  <si>
+    <t>Epoch 020 | lr=9.40e-04 | train_loss=0.3857 | val_loss=0.4619 | val_mIoU=0.1750 | val_mF1=0.2631 | val_acc=0.4453</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.117  cls1=0.000  cls2=0.408</t>
+  </si>
+  <si>
+    <t>Epoch 021 | lr=9.32e-04 | train_loss=0.3719 | val_loss=0.4890 | val_mIoU=0.1911 | val_mF1=0.2898 | val_acc=0.4557</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.180  cls1=0.000  cls2=0.394</t>
+  </si>
+  <si>
+    <t>Epoch 022 | lr=9.24e-04 | train_loss=0.3748 | val_loss=0.4687 | val_mIoU=0.2109 | val_mF1=0.3183 | val_acc=0.4736</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.255  cls1=0.000  cls2=0.377</t>
+  </si>
+  <si>
+    <t>Epoch 023 | lr=9.15e-04 | train_loss=0.3844 | val_loss=0.4691 | val_mIoU=0.2215 | val_mF1=0.3318 | val_acc=0.4850</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.298  cls1=0.000  cls2=0.367</t>
+  </si>
+  <si>
+    <t>Epoch 024 | lr=9.05e-04 | train_loss=0.3748 | val_loss=0.4893 | val_mIoU=0.1933 | val_mF1=0.2941 | val_acc=0.4548</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.195  cls1=0.000  cls2=0.385</t>
+  </si>
+  <si>
+    <t>Epoch 025 | lr=8.96e-04 | train_loss=0.3802 | val_loss=0.4916 | val_mIoU=0.1723 | val_mF1=0.2584 | val_acc=0.4434</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.108  cls1=0.000  cls2=0.409</t>
+  </si>
+  <si>
+    <t>Epoch 026 | lr=8.85e-04 | train_loss=0.3869 | val_loss=0.4999 | val_mIoU=0.1665 | val_mF1=0.2490 | val_acc=0.4370</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.091  cls1=0.000  cls2=0.408</t>
+  </si>
+  <si>
+    <t>Epoch 027 | lr=8.75e-04 | train_loss=0.3777 | val_loss=0.4837 | val_mIoU=0.1534 | val_mF1=0.2270 | val_acc=0.4229</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.055  cls1=0.000  cls2=0.406</t>
+  </si>
+  <si>
+    <t>Epoch 028 | lr=8.64e-04 | train_loss=0.3774 | val_loss=0.5085 | val_mIoU=0.2174 | val_mF1=0.3256 | val_acc=0.4848</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.263  cls1=0.000  cls2=0.389</t>
+  </si>
+  <si>
+    <t>Epoch 029 | lr=8.52e-04 | train_loss=0.3842 | val_loss=0.4742 | val_mIoU=0.1950 | val_mF1=0.2941 | val_acc=0.4642</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.181  cls1=0.000  cls2=0.404</t>
+  </si>
+  <si>
+    <t>Epoch 030 | lr=8.40e-04 | train_loss=0.3638 | val_loss=0.5197 | val_mIoU=0.1890 | val_mF1=0.2865 | val_acc=0.4544</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.171  cls1=0.000  cls2=0.396</t>
+  </si>
+  <si>
+    <t>Epoch 031 | lr=8.28e-04 | train_loss=0.3805 | val_loss=0.5222 | val_mIoU=0.2340 | val_mF1=0.3463 | val_acc=0.5024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         per-class IoU → cls0=0.334  cls1=0.000  cls2=0.368</t>
+  </si>
+  <si>
+    <t>Early stopping triggered after 31 epochs (20 epochs without improvement).</t>
   </si>
 </sst>
 </file>
@@ -1035,4 +1249,379 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A74"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>156</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>